<commit_message>
Regenerate QA Excel in compatible format
</commit_message>
<xml_diff>
--- a/QA_Test_Cases_Bill_Over_45_Days.xlsx
+++ b/QA_Test_Cases_Bill_Over_45_Days.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Requirement Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Requirement" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Date Examples" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -46,7 +54,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -65,37 +73,34 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -172,25 +177,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QATestCases" displayName="QATestCases" ref="A1:J13" headerRowCount="1">
-  <autoFilter ref="A1:J13"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="TC ID"/>
-    <tableColumn id="2" name="Module/Service"/>
-    <tableColumn id="3" name="Scenario"/>
-    <tableColumn id="4" name="Precondition"/>
-    <tableColumn id="5" name="Test Data"/>
-    <tableColumn id="6" name="Test Steps"/>
-    <tableColumn id="7" name="Expected Result"/>
-    <tableColumn id="8" name="Expected Kibana Log"/>
-    <tableColumn id="9" name="Priority"/>
-    <tableColumn id="10" name="Status"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -485,21 +471,26 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="115" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Requirement Summary</t>
+          <t>รายการ</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>รายละเอียด</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>หัวข้อ</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -511,31 +502,31 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>วัตถุประสงค์</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ป้องกันไม่ให้นำบิลขาย/บิลคืนย้อนหลังครบหรือเกิน 45 วัน ไปปรับ Stock และ BOM แต่ต้องมี Log ใน Kibana เพื่อให้ตรวจสอบย้อนหลังได้</t>
+          <t>เช็ค businessDate ของบิลขาย/บิลคืนก่อนนำไปปรับ Stock และ BOM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>วันที่ใช้เทียบ</t>
+          <t>Date Reference</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>วันที่ server ปัจจุบัน</t>
+          <t>เทียบกับวันที่ server ปัจจุบัน</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>วิธีเทียบวันที่</t>
+          <t>Compare Rule</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -547,7 +538,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>เงื่อนไขที่ต้อง Block/Log</t>
+          <t>Block Condition</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -559,55 +550,52 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>เงื่อนไขที่ยังทำงานปกติ</t>
+          <t>Normal Condition</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>businessDate ย้อนหลังน้อยกว่า 45 วัน</t>
+          <t>businessDate ย้อนหลังน้อยกว่า 45 วัน ให้ทำงานตาม flow ปกติ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Service ที่ต้องตรวจสอบ Log</t>
+          <t>Expected Behavior</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Stock service และ BOM service</t>
+          <t>ถ้าเข้าเงื่อนไข 45 วัน: ไม่ปรับ Stock, ไม่ปรับ BOM และมี Log ใน Kibana</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ข้อความ Log ที่คาดหวัง</t>
+          <t>Log Service</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: &lt;branchCode&gt;, billNo: &lt;billNo&gt;</t>
+          <t>แยกตาม service: Stock และ BOM</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Error case อื่น</t>
+          <t>Log Message Format</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>ไม่ต้องแยก error เพิ่มเติมตามข้อมูลที่ยืนยัน</t>
+          <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: &lt;branchCode&gt;, billNo: &lt;billNo&gt;</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -618,95 +606,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>TC ID</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Module/Service</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Step</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Expected Kibana Log</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Kibana Log</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>TC01</t>
-        </is>
+      <c r="A2" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลขายย้อนหลังน้อยกว่า 45 วัน</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>บิลขายย้อนหลังน้อยกว่า 45 วัน</t>
+          <t>ระบบพร้อมรับ sale transaction</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ sale transaction และมีสินค้า/สาขาสำหรับทดสอบ</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>type = SALE
 businessDate = server date - 44 วัน
@@ -714,7 +689,7 @@
 billNo = QA-SALE-44D</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง transaction เข้าระบบ
 2. ตรวจสอบ Stock movement
@@ -722,51 +697,44 @@
 4. ตรวจสอบ Kibana</t>
         </is>
       </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ระบบปรับ Stock/BOM ตาม flow ปกติ
+มี movement ตามรายการ
+ไม่มี log error</t>
+        </is>
+      </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>ระบบส่งไปปรับ Stock/BOM ตาม flow ปกติ
-มี movement เกิดขึ้นตามรายการ
-ไม่มี log businessDate older than 45 days</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>ไม่ควรพบ log error</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
+          <t>ไม่ควรพบ log businessDate is older than 45 days</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>TC02</t>
-        </is>
+      <c r="A3" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลขายย้อนหลังครบ 45 วันพอดี</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>บิลขายย้อนหลังครบ 45 วันพอดี</t>
+          <t>ระบบพร้อมรับ sale transaction</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ sale transaction</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>type = SALE
 businessDate = server date - 45 วัน
@@ -774,59 +742,52 @@
 billNo = QA-SALE-45D</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>1. ส่ง transaction เข้าระบบ
+2. ตรวจสอบ Stock movement
+3. ตรวจสอบ BOM movement
+4. ตรวจสอบ Kibana service Stock/BOM</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1. ส่ง transaction เข้าระบบ
-2. ตรวจสอบว่าไม่มี Stock movement ใหม่
-3. ตรวจสอบว่าไม่มี BOM movement ใหม่
-4. ตรวจสอบ Kibana ทั้ง Stock และ BOM service</t>
+          <t>ไม่ปรับ Stock
+ไม่ปรับ BOM
+ต้องมี log ใน Kibana</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>ระบบไม่ส่งไปปรับ Stock
-ระบบไม่ส่งไปปรับ BOM
-ต้องมี log ใน Kibana</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: M04C, billNo: QA-SALE-45D</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>TC03</t>
-        </is>
+      <c r="A4" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลขายย้อนหลังเกิน 45 วัน</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>บิลขายย้อนหลังเกิน 45 วัน</t>
+          <t>ระบบพร้อมรับ sale transaction</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ sale transaction</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>type = SALE
 businessDate = server date - 46 วัน
@@ -834,59 +795,52 @@
 billNo = QA-SALE-46D</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง transaction เข้าระบบ
 2. ตรวจสอบ Stock movement
 3. ตรวจสอบ BOM movement
-4. ตรวจสอบ Kibana ทั้ง Stock และ BOM service</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>ระบบไม่ส่งไปปรับ Stock/BOM
+4. ตรวจสอบ Kibana service Stock/BOM</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ไม่ปรับ Stock/BOM
 ไม่เกิด movement ใหม่
 ต้องมี log ใน Kibana</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: M04C, billNo: QA-SALE-46D</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>TC04</t>
-        </is>
+      <c r="A5" s="4" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลคืนย้อนหลังน้อยกว่า 45 วัน</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>บิลคืนย้อนหลังน้อยกว่า 45 วัน</t>
+          <t>ระบบพร้อมรับ return transaction</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ return transaction และมี bill reference/สินค้า/สาขาสำหรับทดสอบ</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>type = RETURN
 businessDate = server date - 44 วัน
@@ -894,7 +848,7 @@
 billNo = QA-RETURN-44D</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง return transaction เข้าระบบ
 2. ตรวจสอบ Stock movement
@@ -902,51 +856,44 @@
 4. ตรวจสอบ Kibana</t>
         </is>
       </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>ระบบปรับ Stock/BOM ตาม flow ปกติ
+มี movement ตามรายการ
+ไม่มี log error</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>ระบบส่งไปปรับ Stock/BOM ตาม flow ปกติ
-มี movement เกิดขึ้นตามรายการ
-ไม่มี log businessDate older than 45 days</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>ไม่ควรพบ log error</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
+          <t>ไม่ควรพบ log businessDate is older than 45 days</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>TC05</t>
-        </is>
+      <c r="A6" s="4" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลคืนย้อนหลังครบ 45 วันพอดี</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>บิลคืนย้อนหลังครบ 45 วันพอดี</t>
+          <t>ระบบพร้อมรับ return transaction</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ return transaction</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>type = RETURN
 businessDate = server date - 45 วัน
@@ -954,59 +901,52 @@
 billNo = QA-RETURN-45D</t>
         </is>
       </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1. ส่ง return transaction เข้าระบบ
+2. ตรวจสอบ Stock movement
+3. ตรวจสอบ BOM movement
+4. ตรวจสอบ Kibana service Stock/BOM</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. ส่ง return transaction เข้าระบบ
-2. ตรวจสอบว่าไม่มี Stock movement ใหม่
-3. ตรวจสอบว่าไม่มี BOM movement ใหม่
-4. ตรวจสอบ Kibana ทั้ง Stock และ BOM service</t>
+          <t>ไม่ปรับ Stock
+ไม่ปรับ BOM
+ต้องมี log ใน Kibana</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>ระบบไม่ส่งไปปรับ Stock
-ระบบไม่ส่งไปปรับ BOM
-ต้องมี log ใน Kibana</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: M04C, billNo: QA-RETURN-45D</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>TC06</t>
-        </is>
+      <c r="A7" s="4" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>บิลคืนย้อนหลังเกิน 45 วัน</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>บิลคืนย้อนหลังเกิน 45 วัน</t>
+          <t>ระบบพร้อมรับ return transaction</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>ระบบพร้อมรับ return transaction</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>type = RETURN
 businessDate = server date - 46 วัน
@@ -1014,282 +954,247 @@
 billNo = QA-RETURN-46D</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง return transaction เข้าระบบ
 2. ตรวจสอบ Stock movement
 3. ตรวจสอบ BOM movement
-4. ตรวจสอบ Kibana ทั้ง Stock และ BOM service</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>ระบบไม่ส่งไปปรับ Stock/BOM
+4. ตรวจสอบ Kibana service Stock/BOM</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>ไม่ปรับ Stock/BOM
 ไม่เกิด movement ใหม่
 ต้องมี log ใน Kibana</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: M04C, billNo: QA-RETURN-46D</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>TC07</t>
-        </is>
+      <c r="A8" s="4" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Stock service</t>
+          <t>ตรวจสอบว่าไม่เกิด Stock movement เมื่อเข้าเงื่อนไข</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>ตรวจสอบว่าไม่เกิด Stock movement เมื่อเข้าเงื่อนไข 45 วัน</t>
+          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน</t>
+          <t>ใช้ billNo จาก TC02, TC03, TC05 หรือ TC06</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
+          <t>1. Query/ตรวจสอบ Stock movement ด้วย billNo
+2. เทียบข้อมูลก่อนและหลังส่ง transaction</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ไม่พบ Stock movement ใหม่จาก billNo ที่เข้าเงื่อนไข block/log</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>พบ log ใน Stock service</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ตรวจสอบว่าไม่เกิด BOM movement เมื่อเข้าเงื่อนไข</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน และเกี่ยวข้องกับ BOM</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
           <t>ใช้ billNo จาก TC02, TC03, TC05 หรือ TC06</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>1. Query/ตรวจสอบ collection หรือหน้าจอ Stock movement ด้วย billNo
-2. เทียบก่อน-หลังส่ง transaction</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>ไม่พบ Stock movement ใหม่จาก billNo ที่เข้าเงื่อนไข block/log</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>พบ log ใน Stock service</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1. Query/ตรวจสอบ BOM movement ด้วย billNo
+2. เทียบข้อมูลก่อนและหลังส่ง transaction</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>ไม่พบ BOM movement ใหม่จาก billNo ที่เข้าเงื่อนไข block/log</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>พบ log ใน BOM service</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TC08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>BOM service</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>ตรวจสอบว่าไม่เกิด BOM movement เมื่อเข้าเงื่อนไข 45 วัน</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน และเป็นรายการที่เกี่ยวข้องกับ BOM</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ใช้ billNo จาก TC02, TC03, TC05 หรือ TC06</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>1. Query/ตรวจสอบ collection หรือหน้าจอ BOM movement ด้วย billNo
-2. เทียบก่อน-หลังส่ง transaction</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>ไม่พบ BOM movement ใหม่จาก billNo ที่เข้าเงื่อนไข block/log</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>พบ log ใน BOM service</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>TC09</t>
-        </is>
+      <c r="A10" s="4" t="n">
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Kibana - Stock service</t>
+          <t>ตรวจสอบ Log ใน Kibana ของ Stock service</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>ตรวจสอบ Log ใน Kibana ของ Stock service</t>
+          <t>ส่ง transaction ที่ businessDate ครบ/เกิน 45 วันแล้ว</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>ส่ง transaction ที่ businessDate ครบ/เกิน 45 วันแล้ว</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>businessDate = server date - 45 วัน หรือ -46 วัน
+          <t>businessDate = server date - 45 หรือ -46 วัน
 branchCode = M04C
 billNo = QA-SALE-45D</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>1. เปิด Kibana
 2. Filter service = Stock
 3. Search ด้วย billNo หรือข้อความ businessDate is older than 45 days</t>
         </is>
       </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>พบ log ใน Stock service และมี businessDate, branchCode, billNo ครบ</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>พบ log ใน Stock service และข้อความมี businessDate, branchCode, billNo ครบถ้วน</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: &lt;branchCode&gt;, billNo: &lt;billNo&gt;</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>TC10</t>
-        </is>
+      <c r="A11" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Kibana - BOM service</t>
+          <t>ตรวจสอบ Log ใน Kibana ของ BOM service</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>ตรวจสอบ Log ใน Kibana ของ BOM service</t>
+          <t>ส่ง transaction ที่ businessDate ครบ/เกิน 45 วันแล้ว</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>ส่ง transaction ที่ businessDate ครบ/เกิน 45 วันแล้ว</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>businessDate = server date - 45 วัน หรือ -46 วัน
+          <t>businessDate = server date - 45 หรือ -46 วัน
 branchCode = M04C
 billNo = QA-SALE-45D</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>1. เปิด Kibana
 2. Filter service = BOM
 3. Search ด้วย billNo หรือข้อความ businessDate is older than 45 days</t>
         </is>
       </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>พบ log ใน BOM service และมี businessDate, branchCode, billNo ครบ</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>พบ log ใน BOM service และข้อความมี businessDate, branchCode, billNo ครบถ้วน</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
           <t>businessDate is older than 45 days. businessDate: &lt;businessDate&gt;, branchCode: &lt;branchCode&gt;, billNo: &lt;billNo&gt;</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>TC11</t>
-        </is>
+      <c r="A12" s="4" t="n">
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Stock/BOM</t>
+          <t>ส่ง transaction เดิมซ้ำ/retry สำหรับบิลที่เข้าเงื่อนไข</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>ส่ง transaction เดิมซ้ำ/retry สำหรับบิลที่เข้าเงื่อนไข 45 วัน</t>
+          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน และเคยส่งแล้ว</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน และเคยส่งแล้ว</t>
+          <t>ใช้ billNo เดิมจาก TC02/TC03/TC05/TC06</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>ใช้ billNo เดิมจาก TC02/TC03/TC05/TC06</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง transaction เดิมซ้ำ
 2. ตรวจสอบ Stock movement
@@ -1297,91 +1202,81 @@
 4. ตรวจสอบ Kibana</t>
         </is>
       </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>ไม่เกิด movement ซ้ำ
+ยัง skip การปรับ Stock/BOM
+มี log ตามเงื่อนไข</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>ไม่เกิด movement ซ้ำ
-ระบบยัง skip การปรับ Stock/BOM
-มี log ตามเงื่อนไข</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>พบ log ตามจำนวนครั้งที่ระบบประมวลผล หรือเป็นไปตาม policy retry/log ของระบบ</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
+          <t>พบ log ตาม policy การ retry/log ของระบบ</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>TC12</t>
-        </is>
+      <c r="A13" s="4" t="n">
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>ตรวจสอบ Format ข้อความ Log</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>ตรวจสอบรูปแบบข้อความ Log</t>
+          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>มี transaction ที่ businessDate ครบ/เกิน 45 วัน</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>businessDate = 2026-05-18T10:21:51.474+0700
 branchCode = M04C
 billNo = S2605M04C149-000067</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>1. ส่ง transaction เข้าระบบ
 2. Search log ใน Kibana ด้วย billNo
 3. ตรวจสอบข้อความ log</t>
         </is>
       </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>ข้อความ log ตรงตาม format ที่กำหนด และมีค่าหลักครบ</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>ข้อความ log ตรงตาม format ที่กำหนด และมีค่าหลักครบ</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
           <t>businessDate is older than 45 days. businessDate: 2026-05-18T10:21:51.474+0700, branchCode: M04C, billNo: S2605M04C149-000067</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J13"/>
+  <autoFilter ref="A1:I13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1394,25 +1289,25 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>สมมติ Server Date</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Server Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>businessDate</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>ผลลัพธ์</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>

</xml_diff>